<commit_message>
Candidate signin & Signup Form and Phase 1 completed
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/ManagerReferral_TestCases.xlsx
+++ b/Test Cases/ManagerReferral_TestCases.xlsx
@@ -4,19 +4,18 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="6615"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="6615" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ManagerReferralPage_TestCases" sheetId="1" r:id="rId1"/>
     <sheet name="ManagerReferralReport_TestCases" sheetId="2" r:id="rId2"/>
-    <sheet name="CandidateAuth_TestCases" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="443">
   <si>
     <t>S.No</t>
   </si>
@@ -1553,597 +1552,13 @@
     <t>headerLogo: present; title/label/button/footer text: OK; column headers: Referral date, iTAP Number, Candidate name, Email ID, Mobile number, Aadhaar number present, but "Initial feedback" column header is misspelled "Initital feedback" on the live page.</t>
   </si>
   <si>
-    <t>Verify all UI components are present on the Candidate Sign In page</t>
-  </si>
-  <si>
-    <t>Verifying that Username, Password, the acknowledgment checkbox, Sign in button, Forgot password link, and Create a new one link are all present/locatable</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Locate the Username (Aadhaar Number) field
-3. Locate the Password field
-4. Locate the acknowledgment checkbox
-5. Locate the Sign in button
-6. Locate the Forgot password link
-7. Locate the Create a new one link</t>
-  </si>
-  <si>
-    <t>All 6 components should be present and visible: Username, Password, acknowledgment checkbox, Sign in button, Forgot password link, Create a new one link</t>
-  </si>
-  <si>
-    <t>usernameInput: present; passwordInput: present; acknowledgmentCheckbox: present; signInButton: present; forgotPasswordLink: present; createAccountLink: present.</t>
-  </si>
-  <si>
-    <t>Verify Sign In succeeds with valid, existing credentials</t>
-  </si>
-  <si>
-    <t>Verifying that signing in with a real account's correct Aadhaar Number and Password succeeds and proceeds into the Application Form</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: 989127033381 (existing account), Password: &lt;correct&gt;</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter the existing account's Username and Password
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Sign in should succeed and the candidate should be taken into the Application Form</t>
-  </si>
-  <si>
-    <t>reached Application Form=true</t>
-  </si>
-  <si>
-    <t>Verify Sign In rejects empty Username</t>
-  </si>
-  <si>
-    <t>Verifying that leaving Username blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: (blank), Password: Passw0rd1</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Leave Username blank, enter a Password
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Username should be rejected with a validation message</t>
-  </si>
-  <si>
-    <t>username aria-invalid=true, message="Please enter valid Aadhaar number"</t>
-  </si>
-  <si>
-    <t>Verify Sign In rejects empty Password</t>
-  </si>
-  <si>
-    <t>Verifying that leaving Password blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: 989127033381, Password: (blank)</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter Username, leave Password blank
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Password should be rejected with a validation message</t>
-  </si>
-  <si>
-    <t>password aria-invalid=true</t>
-  </si>
-  <si>
-    <t>Verify Sign In rejects a non-numeric Username</t>
-  </si>
-  <si>
-    <t>Verifying that an alphabetic Username is rejected since Aadhaar Number must be digits only</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: abcdefghijkl</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter Username "abcdefghijkl"
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Verify Sign In rejects a Username shorter than 12 digits</t>
-  </si>
-  <si>
-    <t>Verifying an 11-digit Username is rejected for not matching the required 12-digit Aadhaar length</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: 12345678901 (11 digits)</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter Username "12345678901" (11 digits)
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Username should be rejected with a validation message for not being 12 digits</t>
-  </si>
-  <si>
-    <t>Verify Sign In Username field restricts input beyond 12 digits</t>
-  </si>
-  <si>
-    <t>Verifying the field caps input at the maximum 12-digit Aadhaar length</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: 1234567890123 (13 digits)</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter Username "1234567890123" (13 digits)
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Input should be capped at 12 digits; the resulting value should still be validated (here, no matching account)</t>
-  </si>
-  <si>
-    <t>Typed 13 chars; field held 12 (maxlength=12). modal="×
-Information
-We couldn’t find your account. Please sign up to get started.
-OK"</t>
-  </si>
-  <si>
-    <t>Verify Sign In requires the acknowledgment checkbox</t>
-  </si>
-  <si>
-    <t>Verifying that submitting with valid credentials but an unchecked acknowledgment checkbox is blocked</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: 989127033381, Password: valid, checkbox: unchecked</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter valid Username and Password
-3. Leave the acknowledgment checkbox unchecked
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Form should not sign in; a message should prompt the user to acknowledge the terms</t>
-  </si>
-  <si>
-    <t>modal="×
-Information
-Please acknowledge the terms before signing in
-OK"</t>
-  </si>
-  <si>
-    <t>Verify Sign In shows an appropriate message for a non-existent account</t>
-  </si>
-  <si>
-    <t>Verifying that valid-format credentials for an account that does not exist show a clear "not found" message</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: &lt;freshly generated, guaranteed unused&gt; (valid format, no account)</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter a valid-format Username with no matching account
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>A message should indicate no account was found and suggest signing up</t>
-  </si>
-  <si>
-    <t>modal="×
-Information
-We couldn’t find your account. Please sign up to get started.
-OK"</t>
-  </si>
-  <si>
-    <t>Verify Sign In shows an appropriate message for a wrong password on an existing account</t>
-  </si>
-  <si>
-    <t>Verifying that a correct Username with an incorrect Password is rejected with a clear message, and does not disclose whether the field at fault is username or password</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: 989127033381 (existing), Password: WrongPass9</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter the existing account's Username with an incorrect Password
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>A message should indicate the username or password is incorrect, without signing in</t>
-  </si>
-  <si>
-    <t>modal="×
-Information
-Your Username or Password is incorrect
-OK"</t>
-  </si>
-  <si>
-    <t>Verify Sign In Username field against script/SQL injection input</t>
-  </si>
-  <si>
-    <t>Verifying that the field safely rejects script tags or SQL injection style input without executing or breaking the application</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin | Username: "&lt;script&gt;alert(1)&lt;/script&gt;" / "' OR '1'='1"</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Enter Username as a script tag or SQL injection string
-3. Check the acknowledgment checkbox
-4. Click Sign in</t>
-  </si>
-  <si>
-    <t>Input should be rejected as an invalid Aadhaar format; no script execution or application error should occur</t>
-  </si>
-  <si>
-    <t>username aria-invalid=true, message="Please enter valid Aadhaar number" secondary: username aria-invalid=true, message="Please enter valid Aadhaar number"</t>
-  </si>
-  <si>
-    <t>Verify all UI components are present on the Candidate Sign Up modal</t>
-  </si>
-  <si>
-    <t>Verifying that Aadhaar Number, Email, New Password, Confirm Password, Manager Reference ID, the acknowledgment checkbox, Sign Up button, close button, and the Sign In toggle link are all present/locatable</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; click "Create a new one"</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Click "Create a new one" to open the Sign Up modal
-3. Locate the Aadhaar Number field
-4. Locate the Email field
-5. Locate the New Password - Mankind ID field
-6. Locate the Confirm Password - Mankind ID field
-7. Locate the Manager Reference ID field
-8. Locate the acknowledgment checkbox
-9. Locate the Sign Up button
-10. Locate the close (X) button
-11. Locate the "Already have an account? Sign In" link</t>
-  </si>
-  <si>
-    <t>All 9 components should be present and visible in the Sign Up modal: Aadhaar Number, Email, New Password, Confirm Password, Manager Reference ID, acknowledgment checkbox, Sign Up button, close button, Sign In toggle link</t>
-  </si>
-  <si>
-    <t>aadhaarNumberInput: present; emailInput: present; newPasswordInput: present; confirmPasswordInput: present; managerReferenceIdInput: present; signUpAcknowledgmentCheckbox: present; signUpButton: present; signUpCloseButton: present; signUpToSignInLink: present.</t>
-  </si>
-  <si>
-    <t>Verify Sign Up succeeds with fully valid data and proceeds to the Application Form</t>
-  </si>
-  <si>
-    <t>Verifying that a fresh Aadhaar Number/Email, a policy-compliant matching password, and a valid Manager Reference ID together complete Sign Up</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Aadhaar: &lt;fresh&gt;, Email: &lt;fresh&gt;, Password: Passw0rd1, Reference ID: 10001556</t>
-  </si>
-  <si>
-    <t>1. Open the candidate login link
-2. Click Create a new one
-3. Enter a fresh Aadhaar Number and Email
-4. Enter matching, policy-compliant New/Confirm Password
-5. Enter Reference ID "10001556"
-6. Check the acknowledgment checkbox
-7. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Sign Up should succeed and the candidate should be taken into the Application Form</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects empty Aadhaar Number</t>
-  </si>
-  <si>
-    <t>Verifying that leaving Aadhaar Number blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Aadhaar: (blank), other fields valid</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Leave Aadhaar Number blank, fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Aadhaar Number should be rejected with a validation message</t>
-  </si>
-  <si>
-    <t>aadhaar aria-invalid=true, message="Enter Valid Aadhaar Number"</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects empty Email</t>
-  </si>
-  <si>
-    <t>Verifying that leaving Email blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Email: (blank), other fields valid</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Leave Email blank, fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Email should be rejected with "Enter Email ID"</t>
-  </si>
-  <si>
-    <t>email aria-invalid=true, message="Enter Email ID"</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects empty New Password</t>
-  </si>
-  <si>
-    <t>Verifying that leaving New Password blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | New Password: (blank), other fields valid</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Leave New Password blank, fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>New Password should be rejected with "Enter Password"</t>
-  </si>
-  <si>
-    <t>newPassword aria-invalid=true</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects empty Confirm Password</t>
-  </si>
-  <si>
-    <t>Verifying that leaving Confirm Password blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Confirm Password: (blank), other fields valid</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Leave Confirm Password blank, fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Confirm Password should be rejected with "Enter Password"</t>
-  </si>
-  <si>
-    <t>confirmPassword aria-invalid=true</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects empty Manager Reference ID</t>
-  </si>
-  <si>
-    <t>Verifying that leaving Manager Reference ID blank is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Reference ID: (blank), other fields valid</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Leave Manager Reference ID blank, fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Manager Reference ID should be rejected mentioning the Division Code</t>
-  </si>
-  <si>
-    <t>referenceId aria-invalid=true, message="Manager Reference ID does not contain the Division Code. Please contact your referrer."</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects a non-numeric Aadhaar Number</t>
-  </si>
-  <si>
-    <t>Verifying that an alphabetic Aadhaar Number is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Aadhaar: abcdefghijkl</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter Aadhaar Number "abcdefghijkl", fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects an Aadhaar Number shorter than 12 digits</t>
-  </si>
-  <si>
-    <t>Verifying an 11-digit Aadhaar Number is rejected for not matching the required length</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Aadhaar: 12345678901 (11 digits)</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter Aadhaar Number "12345678901" (11 digits), fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Aadhaar Number should be rejected with a validation message for not being 12 digits</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects an invalid Email format</t>
-  </si>
-  <si>
-    <t>Verifying that a malformed email address is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Email: notanemail</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter Email "notanemail", fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Email should be rejected with "Please enter a valid email address."</t>
-  </si>
-  <si>
-    <t>email aria-invalid=true, message="Please enter a valid email address."</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects a New Password with no digit</t>
-  </si>
-  <si>
-    <t>Verifying the password policy (8 chars + at least 1 digit) rejects an all-letters password</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | New/Confirm Password: Password (no digit)</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter New/Confirm Password "Password" (8 letters, no digit), fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>A password policy modal should be shown: "Check Password policy 8 Character and at least 1 digit should be there."</t>
-  </si>
-  <si>
-    <t>modal="×
-Information
-Check Password policy 8 Character and at least 1 digit should be there.
-OK"</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects a New Password shorter than 8 characters</t>
-  </si>
-  <si>
-    <t>Verifying the password policy rejects a password shorter than the minimum 8 characters</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | New/Confirm Password: Pass1 (5 chars)</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter New/Confirm Password "Pass1" (5 chars), fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>The same password policy modal should be shown for a too-short password</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects a mismatched Confirm Password</t>
-  </si>
-  <si>
-    <t>Verifying that a Confirm Password different from New Password is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | New Password: Passw0rd1, Confirm Password: Passw0rd2</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter different, both policy-valid New Password and Confirm Password
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Confirm Password should be rejected with "New Password and Confirm Password must be same"</t>
-  </si>
-  <si>
-    <t>confirmPassword aria-invalid=true, message="New Password and Confirm Password must be same"</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects a well-formed but unmatched Manager Reference ID</t>
-  </si>
-  <si>
-    <t>Verifying an 8-digit code that is not a real/matching SAP code is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Reference ID: 99999999 (valid shape, not a real code)</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter Reference ID "99999999" (8 digits, not a real code), fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Manager Reference ID should be rejected, directing the candidate to verify it with their referring manager</t>
-  </si>
-  <si>
-    <t>referenceId aria-invalid=true, message="Please enter correct Manager Reference ID as provided by your referring manager or refer to the Sign-up email that you have received"</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects a non-numeric Manager Reference ID</t>
-  </si>
-  <si>
-    <t>Verifying a non-numeric Reference ID is rejected the same way as a well-formed-but-unmatched one</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Reference ID: abcd1234</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter Reference ID "abcd1234", fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Manager Reference ID should be rejected the same way as a well-formed but unmatched code</t>
-  </si>
-  <si>
-    <t>Verify Sign Up requires the acknowledgment checkbox</t>
-  </si>
-  <si>
-    <t>Verifying that submitting with otherwise-valid data but an unchecked acknowledgment checkbox is blocked</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | all fields valid, checkbox unchecked</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Fill every field validly
-3. Leave the acknowledgment checkbox unchecked
-4. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Form should not sign up; a message should prompt the user to acknowledge the terms</t>
-  </si>
-  <si>
-    <t>Verify Sign Up rejects an already-registered Aadhaar Number</t>
-  </si>
-  <si>
-    <t>Verifying that signing up again with an Aadhaar Number that already has an account is rejected</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Aadhaar: 989127033381 (already registered)</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter the already-registered Aadhaar Number with a fresh Email
-3. Fill remaining fields validly
-4. Click Sign Up</t>
-  </si>
-  <si>
-    <t>A message should indicate an account with this Aadhaar number already exists</t>
-  </si>
-  <si>
-    <t>modal="×
-Information
-An account with this aadhaar number already exists. Please log in or use the ‘Forgot Password’ option to reset your credentials.
-OK"</t>
-  </si>
-  <si>
-    <t>Verify Sign Up Email field against script/SQL injection input</t>
-  </si>
-  <si>
-    <t>link: https://fcadmin100-dev.apps.ap-3a.mendixcloud.com/p/candidatelogin -&gt; Create a new one | Email: "&lt;script&gt;alert(1)&lt;/script&gt;" / "' OR '1'='1"</t>
-  </si>
-  <si>
-    <t>1. Open Sign Up
-2. Enter Email as a script tag or SQL injection string, fill other fields validly
-3. Click Sign Up</t>
-  </si>
-  <si>
-    <t>Input should be rejected as an invalid email format; no script execution or application error should occur</t>
-  </si>
-  <si>
-    <t>email aria-invalid=true, message="Please enter a valid email address." secondary: email aria-invalid=true, message="Please enter a valid email address."</t>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
   </si>
 </sst>
 </file>
@@ -2493,7 +1908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.140625" style="1" customWidth="1"/>
@@ -2510,7 +1925,7 @@
     <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2541,8 +1956,11 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K1" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2574,7 +1992,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -2605,8 +2023,11 @@
       <c r="J3" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K3" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2638,7 +2059,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2670,7 +2091,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2702,7 +2123,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2734,7 +2155,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2766,7 +2187,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2798,7 +2219,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2830,7 +2251,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2862,7 +2283,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2894,7 +2315,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2926,7 +2347,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>14</v>
       </c>
@@ -2958,7 +2379,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>15</v>
       </c>
@@ -2990,7 +2411,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>16</v>
       </c>
@@ -3022,7 +2443,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>17</v>
       </c>
@@ -3054,7 +2475,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>18</v>
       </c>
@@ -3086,7 +2507,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>19</v>
       </c>
@@ -3118,7 +2539,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:10" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>20</v>
       </c>
@@ -3149,8 +2570,11 @@
       <c r="J20" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K20" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>21</v>
       </c>
@@ -3181,8 +2605,11 @@
       <c r="J21" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K21" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>22</v>
       </c>
@@ -3214,7 +2641,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>23</v>
       </c>
@@ -3246,7 +2673,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>24</v>
       </c>
@@ -3278,7 +2705,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>25</v>
       </c>
@@ -3310,7 +2737,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>26</v>
       </c>
@@ -3342,7 +2769,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>27</v>
       </c>
@@ -3374,7 +2801,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>28</v>
       </c>
@@ -3406,7 +2833,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>29</v>
       </c>
@@ -3438,7 +2865,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>30</v>
       </c>
@@ -3470,7 +2897,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>31</v>
       </c>
@@ -3502,7 +2929,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>32</v>
       </c>
@@ -3534,7 +2961,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>33</v>
       </c>
@@ -3566,7 +2993,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>34</v>
       </c>
@@ -3598,7 +3025,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:10" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>35</v>
       </c>
@@ -3629,8 +3056,11 @@
       <c r="J35" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K35" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>36</v>
       </c>
@@ -3661,8 +3091,11 @@
       <c r="J36" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K36" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>37</v>
       </c>
@@ -3694,7 +3127,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>38</v>
       </c>
@@ -3726,7 +3159,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>39</v>
       </c>
@@ -3758,7 +3191,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>40</v>
       </c>
@@ -3790,7 +3223,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>41</v>
       </c>
@@ -3822,7 +3255,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>42</v>
       </c>
@@ -3854,7 +3287,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>43</v>
       </c>
@@ -3886,7 +3319,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>44</v>
       </c>
@@ -3918,7 +3351,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>45</v>
       </c>
@@ -3950,7 +3383,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>46</v>
       </c>
@@ -3982,7 +3415,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>47</v>
       </c>
@@ -4014,7 +3447,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>48</v>
       </c>
@@ -4206,7 +3639,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="225" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="225" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -4246,7 +3679,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1" customWidth="1"/>
@@ -4261,7 +3694,7 @@
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4292,8 +3725,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -4325,7 +3761,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -4357,7 +3793,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -4389,7 +3825,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -4421,7 +3857,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -4453,7 +3889,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -4485,7 +3921,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -4517,7 +3953,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -4549,7 +3985,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="210" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -4581,7 +4017,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -4613,7 +4049,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -4645,7 +4081,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -4677,7 +4113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -4709,7 +4145,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -4741,7 +4177,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -4773,7 +4209,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:10" s="4" customFormat="1" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" s="4" customFormat="1" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -4805,7 +4241,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="210" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -4837,7 +4273,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:10" s="3" customFormat="1" ht="165" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" s="3" customFormat="1" ht="165" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -4868,989 +4304,8 @@
       <c r="J19" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="9.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="50" style="1" customWidth="1"/>
-    <col min="7" max="7" width="45.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="44.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="55.85546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="K19" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>444</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>450</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>469</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>477</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>480</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>483</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>489</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>494</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>495</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>11</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>503</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>509</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>510</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>511</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>14</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>514</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>515</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>517</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>518</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>519</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>15</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>520</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>521</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>16</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>527</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>529</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>530</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>531</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>17</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>532</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>536</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>537</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>18</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>538</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>539</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>542</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>545</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>546</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>518</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>519</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>20</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>548</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>549</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>550</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>552</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>519</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>21</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>553</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>554</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>556</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>557</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>22</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>559</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>561</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>562</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>563</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>23</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>565</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>566</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>567</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>568</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>569</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>24</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>571</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>575</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>25</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>576</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>577</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>578</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>579</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>580</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>26</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>582</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>583</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>584</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>585</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>586</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>27</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>588</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>591</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>28</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>593</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>594</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>595</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>596</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>597</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>29</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>599</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>601</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>602</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>